<commit_message>
Reconciliation legend: calculator confirmed correct
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ksw4wYjJxTxvwP8pELDevL
</commit_message>
<xml_diff>
--- a/コミッション照合_2026年10月.xlsx
+++ b/コミッション照合_2026年10月.xlsx
@@ -252,7 +252,7 @@
     <t xml:space="preserve">詳細</t>
   </si>
   <si>
-    <t xml:space="preserve">要判断・確認</t>
+    <t xml:space="preserve">判定</t>
   </si>
   <si>
     <t xml:space="preserve">Goo Property Singapore Pte. Ltd.</t>
@@ -4524,7 +4524,65 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">推薦者コード管理の区分次第。区分が正しければ計算表が正。要判断の推薦者は区分を確認してください。</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">計算表（推薦者コード管理の区分が正しいと確認済み </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026/10/18</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）。管理シート</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">一覧は平準の人も</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">×12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">で計上しており誤り。</t>
+    </r>
   </si>
   <si>
     <r>
@@ -17946,7 +18004,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
         <v>252</v>
       </c>

</xml_diff>